<commit_message>
Ajustes reportes y endosos de fianzas
</commit_message>
<xml_diff>
--- a/importaciones/UNICA import  - UAT.xlsx
+++ b/importaciones/UNICA import  - UAT.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{64B2C7A5-7851-4808-A58A-C9BB12AF6F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5E5DD18-5963-4272-BCFE-A3BF8EBECF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UNICA import  - UAT" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="25">
   <si>
     <t>casegurado</t>
   </si>
@@ -73,9 +73,6 @@
     <t>Cob_169_Suma Asegurada</t>
   </si>
   <si>
-    <t>Trimestral</t>
-  </si>
-  <si>
     <t>CPR</t>
   </si>
   <si>
@@ -85,22 +82,25 @@
     <t>S</t>
   </si>
   <si>
-    <t>m</t>
-  </si>
-  <si>
     <t>ACH</t>
   </si>
   <si>
-    <t>Contado</t>
-  </si>
-  <si>
     <t>PRO</t>
+  </si>
+  <si>
+    <t>01/09/2026</t>
+  </si>
+  <si>
+    <t>30/09/2026</t>
+  </si>
+  <si>
+    <t>Pago Único</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -237,7 +237,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -415,6 +415,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -578,9 +584,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="33" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -935,7 +943,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1014,37 +1022,31 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="1">
-        <v>46266</v>
-      </c>
-      <c r="G2" s="1">
-        <v>46295</v>
+      <c r="F2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="H2">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="I2">
         <v>3200</v>
       </c>
       <c r="M2" t="s">
+        <v>18</v>
+      </c>
+      <c r="N2" t="s">
         <v>19</v>
       </c>
-      <c r="N2" t="s">
-        <v>20</v>
-      </c>
-      <c r="O2">
-        <v>15000</v>
-      </c>
       <c r="P2" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q2">
-        <v>15000</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -1058,69 +1060,63 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="1">
-        <v>46266</v>
-      </c>
-      <c r="G3" s="1">
-        <v>46295</v>
+      <c r="G3" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="H3">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="N3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="P3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
+    <row r="4" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2">
         <v>1</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I4" s="2">
+        <v>3200</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="1">
-        <v>46266</v>
-      </c>
-      <c r="G4" s="1">
-        <v>46295</v>
-      </c>
-      <c r="H4">
-        <v>15000</v>
-      </c>
-      <c r="I4">
-        <v>3200</v>
-      </c>
-      <c r="M4" t="s">
+      <c r="N4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="N4" t="s">
-        <v>20</v>
-      </c>
-      <c r="O4">
-        <v>15000</v>
-      </c>
-      <c r="P4" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q4">
-        <v>15000</v>
+      <c r="P4" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -1134,28 +1130,29 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="1">
-        <v>46266</v>
-      </c>
-      <c r="G5" s="1">
-        <v>46295</v>
-      </c>
       <c r="H5">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="N5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="P5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>